<commit_message>
v1.14.3: formato condicional sku/link y guía de tallas por defecto, editable en la vista previa
</commit_message>
<xml_diff>
--- a/plantilla.xlsx
+++ b/plantilla.xlsx
@@ -17495,29 +17495,14 @@
       <c r="L1000" s="10"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F1000">
+  <conditionalFormatting sqref="B2:B1000">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND($A2="Sephora", $F2="")</formula>
+      <formula>OR(AND($A2="Amazon", $B2=""), AND($A2&lt;&gt;"", $A2&lt;&gt;"Amazon", $B2&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B1000">
+  <conditionalFormatting sqref="F2:F1000">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND($A2="Amazon", $B2="")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B1000">
-    <cfRule type="expression" dxfId="0" priority="3">
-      <formula>AND($A2="Marc Jacobs", $B2="")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B1000">
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>AND($A2="Kate Spade", $B2="")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B1000">
-    <cfRule type="expression" dxfId="0" priority="5">
-      <formula>AND($A2="Michael Kors", $B2="")</formula>
+      <formula>OR(AND($A2&lt;&gt;"", $A2&lt;&gt;"Amazon", $F2=""), AND($A2="Amazon", $F2&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
@@ -17527,8 +17512,11 @@
     <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="G2:G1000">
       <formula1>Mapeo_categorias!$E$2:$E$2000</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" prompt="Link obligatorio si ecommerce es Sephora" sqref="F2:F1000">
-      <formula1>OR($A2&lt;&gt;"Sephora", $F2&lt;&gt;"")</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Link obligatorio si el ecommerce no es Amazon (Amazon va sin link)" sqref="F2:F1000">
+      <formula1>OR($A2="Amazon", $A2="", $F2&lt;&gt;"")</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" prompt="sku obligatorio solo si el ecommerce es Amazon (los demás van sin sku)" sqref="B2:B1000">
+      <formula1>OR($A2&lt;&gt;"Amazon", $B2&lt;&gt;"")</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E1000">
       <formula1>"Nuevo,Reacondicionado"</formula1>

</xml_diff>